<commit_message>
update agent headoffice excel file
</commit_message>
<xml_diff>
--- a/Jobs/Tasks/FileProcess/TempFile_HO.xlsx
+++ b/Jobs/Tasks/FileProcess/TempFile_HO.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="201">
   <si>
     <t>AgentName</t>
   </si>
@@ -616,9 +616,6 @@
   </si>
   <si>
     <t>Head Office</t>
-  </si>
-  <si>
-    <t>Agency Head Office</t>
   </si>
   <si>
     <t>Tim Murphy</t>
@@ -1576,14 +1573,14 @@
     </row>
     <row r="2" spans="1:133" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B2" t="str">
         <f>TRIM(A2)</f>
         <v>Tim Murphy</v>
       </c>
       <c r="C2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D2" t="s">
         <v>167</v>
@@ -1943,7 +1940,7 @@
         <v>156</v>
       </c>
       <c r="EC2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
   </sheetData>

</xml_diff>